<commit_message>
switch age groups to 2025
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/agegroups/AgeGroups.xlsx
+++ b/owlcms/src/main/resources/agegroups/AgeGroups.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\agegroups\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C697D50-5764-478D-9AFF-0855A426BDCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CB18353-63C4-42CC-9BD3-F86E967A9CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2430" yWindow="2685" windowWidth="24615" windowHeight="11310" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AgeGroups" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="77">
   <si>
     <t>code</t>
   </si>
@@ -57,12 +57,6 @@
     <t>active</t>
   </si>
   <si>
-    <t>#bodyweight categories or each age group (bodyweight category code followed by optional qualifying total, example: 45 80)</t>
-  </si>
-  <si>
-    <t>U10</t>
-  </si>
-  <si>
     <t>U</t>
   </si>
   <si>
@@ -207,10 +201,70 @@
     <t>agegroupscoring</t>
   </si>
   <si>
-    <t>QPOINTS</t>
+    <t>48</t>
+  </si>
+  <si>
+    <t>53</t>
+  </si>
+  <si>
+    <t>63</t>
+  </si>
+  <si>
+    <t>69</t>
+  </si>
+  <si>
+    <t>77</t>
+  </si>
+  <si>
+    <t>86</t>
+  </si>
+  <si>
+    <t>58</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>65</t>
+  </si>
+  <si>
+    <t>71</t>
+  </si>
+  <si>
+    <t>88</t>
+  </si>
+  <si>
+    <t>110</t>
+  </si>
+  <si>
+    <t>79</t>
+  </si>
+  <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>U11</t>
+  </si>
+  <si>
+    <t>U23</t>
+  </si>
+  <si>
+    <t>56</t>
+  </si>
+  <si>
+    <t>44</t>
   </si>
   <si>
     <t>agegroupbestathlete</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>QPoints</t>
   </si>
 </sst>
 </file>
@@ -256,7 +310,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -267,6 +321,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF8EA9DB"/>
         <bgColor rgb="FF969696"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -282,7 +342,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -305,6 +365,7 @@
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -572,9 +633,10 @@
     <col min="1" max="1" width="14.42578125" customWidth="1"/>
     <col min="2" max="2" width="16.85546875" style="1" customWidth="1"/>
     <col min="3" max="7" width="14.42578125" customWidth="1"/>
-    <col min="8" max="9" width="21.85546875" customWidth="1"/>
-    <col min="10" max="23" width="14.42578125" style="1" customWidth="1"/>
-    <col min="24" max="28" width="14.42578125" customWidth="1"/>
+    <col min="8" max="8" width="16.7109375" customWidth="1"/>
+    <col min="9" max="9" width="20.7109375" customWidth="1"/>
+    <col min="10" max="22" width="14.42578125" style="1" customWidth="1"/>
+    <col min="23" max="27" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -600,14 +662,12 @@
         <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>56</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>7</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="I1" t="s">
+        <v>74</v>
+      </c>
+      <c r="J1" s="5"/>
       <c r="K1" s="5"/>
       <c r="L1" s="5"/>
       <c r="M1" s="5"/>
@@ -620,20 +680,19 @@
       <c r="T1" s="5"/>
       <c r="U1" s="5"/>
       <c r="V1" s="5"/>
-      <c r="W1" s="5"/>
     </row>
     <row r="2" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E2" s="7">
         <v>0</v>
@@ -644,13 +703,10 @@
       <c r="G2" s="8" t="b">
         <v>0</v>
       </c>
-      <c r="H2" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="I2" s="8"/>
-      <c r="J2" s="6" t="s">
-        <v>53</v>
-      </c>
+      <c r="H2" t="s">
+        <v>76</v>
+      </c>
+      <c r="J2" s="6"/>
       <c r="K2" s="6"/>
       <c r="L2" s="6"/>
       <c r="M2" s="6"/>
@@ -663,42 +719,54 @@
       <c r="T2" s="6"/>
       <c r="U2" s="6"/>
       <c r="V2" s="6"/>
-      <c r="W2" s="6"/>
     </row>
     <row r="3" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="E3" s="7">
         <v>0</v>
       </c>
       <c r="F3" s="7">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G3" s="8" t="b">
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="6">
-        <v>999</v>
-      </c>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="6"/>
-      <c r="P3" s="6"/>
+      <c r="H3" t="s">
+        <v>75</v>
+      </c>
+      <c r="J3" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N3" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P3" s="6" t="s">
+        <v>51</v>
+      </c>
       <c r="Q3" s="6"/>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
@@ -709,16 +777,16 @@
     </row>
     <row r="4" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E4" s="7">
         <v>11</v>
@@ -730,35 +798,34 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="6">
-        <v>35</v>
-      </c>
-      <c r="K4" s="6">
-        <v>40</v>
-      </c>
-      <c r="L4" s="6">
-        <v>45</v>
-      </c>
-      <c r="M4" s="6">
-        <v>49</v>
-      </c>
-      <c r="N4" s="6">
+      <c r="H4" t="s">
+        <v>75</v>
+      </c>
+      <c r="J4" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="L4" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O4" s="6">
-        <v>59</v>
-      </c>
-      <c r="P4" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q4" s="6">
-        <v>71</v>
-      </c>
-      <c r="R4" s="6">
-        <v>999</v>
-      </c>
+      <c r="M4" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N4" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O4" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P4" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q4" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="R4" s="6"/>
       <c r="S4" s="6"/>
       <c r="T4" s="6"/>
       <c r="U4" s="6"/>
@@ -767,16 +834,16 @@
     </row>
     <row r="5" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E5" s="7">
         <v>14</v>
@@ -788,38 +855,35 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="6">
-        <v>35</v>
-      </c>
-      <c r="K5" s="6">
-        <v>40</v>
-      </c>
-      <c r="L5" s="6">
-        <v>45</v>
-      </c>
-      <c r="M5" s="6">
-        <v>49</v>
-      </c>
-      <c r="N5" s="6">
+      <c r="H5" t="s">
+        <v>75</v>
+      </c>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="L5" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O5" s="6">
+      <c r="M5" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N5" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O5" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P5" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q5" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P5" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q5" s="6">
-        <v>71</v>
-      </c>
-      <c r="R5" s="6">
-        <v>76</v>
-      </c>
-      <c r="S5" s="6">
-        <v>999</v>
-      </c>
+      <c r="R5" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="S5" s="6"/>
       <c r="T5" s="6"/>
       <c r="U5" s="6"/>
       <c r="V5" s="6"/>
@@ -827,16 +891,16 @@
     </row>
     <row r="6" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E6" s="7">
         <v>16</v>
@@ -848,55 +912,52 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
+      <c r="H6" t="s">
+        <v>75</v>
+      </c>
       <c r="J6" s="6"/>
-      <c r="K6" s="6">
-        <v>40</v>
-      </c>
-      <c r="L6" s="6">
-        <v>45</v>
-      </c>
-      <c r="M6" s="6">
-        <v>49</v>
-      </c>
-      <c r="N6" s="6">
+      <c r="K6" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="L6" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O6" s="6">
+      <c r="M6" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O6" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P6" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q6" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P6" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q6" s="6">
-        <v>71</v>
-      </c>
-      <c r="R6" s="6">
-        <v>76</v>
-      </c>
-      <c r="S6" s="6">
-        <v>81</v>
-      </c>
-      <c r="T6" s="6">
-        <v>999</v>
-      </c>
+      <c r="R6" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="S6" s="6"/>
+      <c r="T6" s="6"/>
       <c r="U6" s="6"/>
       <c r="V6" s="6"/>
       <c r="W6" s="6"/>
     </row>
     <row r="7" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E7" s="7">
         <v>18</v>
@@ -908,115 +969,109 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
+      <c r="H7" t="s">
+        <v>75</v>
+      </c>
       <c r="J7" s="6"/>
       <c r="K7" s="6"/>
-      <c r="L7" s="6">
-        <v>45</v>
-      </c>
-      <c r="M7" s="6">
-        <v>49</v>
-      </c>
-      <c r="N7" s="6">
+      <c r="L7" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O7" s="6">
+      <c r="M7" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N7" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O7" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P7" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q7" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P7" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q7" s="6">
-        <v>71</v>
-      </c>
-      <c r="R7" s="6">
-        <v>76</v>
-      </c>
-      <c r="S7" s="6">
-        <v>81</v>
-      </c>
-      <c r="T7" s="6">
-        <v>87</v>
-      </c>
-      <c r="U7" s="6">
-        <v>999</v>
-      </c>
+      <c r="R7" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="S7" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
       <c r="V7" s="6"/>
       <c r="W7" s="6"/>
     </row>
     <row r="8" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E8" s="7">
         <v>21</v>
       </c>
       <c r="F8" s="7">
-        <v>999</v>
+        <v>23</v>
       </c>
       <c r="G8" s="8" t="b">
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
+      <c r="H8" t="s">
+        <v>75</v>
+      </c>
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
-      <c r="L8" s="6">
-        <v>45</v>
-      </c>
-      <c r="M8" s="6">
-        <v>49</v>
-      </c>
-      <c r="N8" s="6">
+      <c r="L8" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O8" s="6">
+      <c r="M8" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N8" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O8" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P8" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q8" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P8" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q8" s="6">
-        <v>71</v>
-      </c>
-      <c r="R8" s="6">
-        <v>76</v>
-      </c>
-      <c r="S8" s="6">
-        <v>81</v>
-      </c>
-      <c r="T8" s="6">
-        <v>87</v>
-      </c>
-      <c r="U8" s="6">
-        <v>999</v>
-      </c>
+      <c r="R8" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="S8" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="T8" s="6"/>
+      <c r="U8" s="6"/>
       <c r="V8" s="6"/>
       <c r="W8" s="6"/>
     </row>
     <row r="9" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="D9" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E9" s="7">
         <v>30</v>
@@ -1028,55 +1083,52 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
+      <c r="H9" t="s">
+        <v>75</v>
+      </c>
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
-      <c r="L9" s="6">
-        <v>45</v>
-      </c>
-      <c r="M9" s="6">
-        <v>49</v>
-      </c>
-      <c r="N9" s="6">
+      <c r="L9" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O9" s="6">
+      <c r="M9" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N9" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O9" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P9" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q9" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P9" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q9" s="6">
-        <v>71</v>
-      </c>
-      <c r="R9" s="6">
-        <v>76</v>
-      </c>
-      <c r="S9" s="6">
-        <v>81</v>
-      </c>
-      <c r="T9" s="6">
-        <v>87</v>
-      </c>
-      <c r="U9" s="6">
-        <v>999</v>
-      </c>
+      <c r="R9" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="S9" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="T9" s="6"/>
+      <c r="U9" s="6"/>
       <c r="V9" s="6"/>
       <c r="W9" s="6"/>
     </row>
     <row r="10" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E10" s="7">
         <v>35</v>
@@ -1088,55 +1140,49 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
-      <c r="L10" s="6">
-        <v>45</v>
-      </c>
-      <c r="M10" s="6">
-        <v>49</v>
-      </c>
-      <c r="N10" s="6">
+      <c r="L10" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O10" s="6">
+      <c r="M10" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N10" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O10" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P10" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q10" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P10" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q10" s="6">
-        <v>71</v>
-      </c>
-      <c r="R10" s="6">
-        <v>76</v>
-      </c>
-      <c r="S10" s="6">
-        <v>81</v>
-      </c>
-      <c r="T10" s="6">
-        <v>87</v>
-      </c>
-      <c r="U10" s="6">
-        <v>999</v>
-      </c>
+      <c r="R10" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="S10" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="T10" s="6"/>
+      <c r="U10" s="6"/>
       <c r="V10" s="6"/>
       <c r="W10" s="6"/>
     </row>
     <row r="11" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E11" s="7">
         <v>40</v>
@@ -1148,55 +1194,49 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
-      <c r="L11" s="6">
-        <v>45</v>
-      </c>
-      <c r="M11" s="6">
-        <v>49</v>
-      </c>
-      <c r="N11" s="6">
+      <c r="L11" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O11" s="6">
+      <c r="M11" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N11" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O11" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P11" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q11" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P11" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q11" s="6">
-        <v>71</v>
-      </c>
-      <c r="R11" s="6">
-        <v>76</v>
-      </c>
-      <c r="S11" s="6">
-        <v>81</v>
-      </c>
-      <c r="T11" s="6">
-        <v>87</v>
-      </c>
-      <c r="U11" s="6">
-        <v>999</v>
-      </c>
+      <c r="R11" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="S11" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="T11" s="6"/>
+      <c r="U11" s="6"/>
       <c r="V11" s="6"/>
       <c r="W11" s="6"/>
     </row>
     <row r="12" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E12" s="7">
         <v>45</v>
@@ -1208,55 +1248,52 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
+      <c r="H12" t="s">
+        <v>75</v>
+      </c>
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
-      <c r="L12" s="6">
-        <v>45</v>
-      </c>
-      <c r="M12" s="6">
-        <v>49</v>
-      </c>
-      <c r="N12" s="6">
+      <c r="L12" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O12" s="6">
+      <c r="M12" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N12" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O12" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P12" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q12" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P12" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q12" s="6">
-        <v>71</v>
-      </c>
-      <c r="R12" s="6">
-        <v>76</v>
-      </c>
-      <c r="S12" s="6">
-        <v>81</v>
-      </c>
-      <c r="T12" s="6">
-        <v>87</v>
-      </c>
-      <c r="U12" s="6">
-        <v>999</v>
-      </c>
+      <c r="R12" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="S12" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="T12" s="6"/>
+      <c r="U12" s="6"/>
       <c r="V12" s="6"/>
       <c r="W12" s="6"/>
     </row>
     <row r="13" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E13" s="7">
         <v>50</v>
@@ -1268,55 +1305,52 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
+      <c r="H13" t="s">
+        <v>75</v>
+      </c>
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
-      <c r="L13" s="6">
-        <v>45</v>
-      </c>
-      <c r="M13" s="6">
-        <v>49</v>
-      </c>
-      <c r="N13" s="6">
+      <c r="L13" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O13" s="6">
+      <c r="M13" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N13" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O13" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P13" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q13" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P13" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q13" s="6">
-        <v>71</v>
-      </c>
-      <c r="R13" s="6">
-        <v>76</v>
-      </c>
-      <c r="S13" s="6">
-        <v>81</v>
-      </c>
-      <c r="T13" s="6">
-        <v>87</v>
-      </c>
-      <c r="U13" s="6">
-        <v>999</v>
-      </c>
+      <c r="R13" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="S13" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="T13" s="6"/>
+      <c r="U13" s="6"/>
       <c r="V13" s="6"/>
       <c r="W13" s="6"/>
     </row>
     <row r="14" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E14" s="7">
         <v>55</v>
@@ -1328,55 +1362,52 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
+      <c r="H14" t="s">
+        <v>75</v>
+      </c>
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
-      <c r="L14" s="6">
-        <v>45</v>
-      </c>
-      <c r="M14" s="6">
-        <v>49</v>
-      </c>
-      <c r="N14" s="6">
+      <c r="L14" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O14" s="6">
+      <c r="M14" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N14" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O14" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P14" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q14" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P14" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q14" s="6">
-        <v>71</v>
-      </c>
-      <c r="R14" s="6">
-        <v>76</v>
-      </c>
-      <c r="S14" s="6">
-        <v>81</v>
-      </c>
-      <c r="T14" s="6">
-        <v>87</v>
-      </c>
-      <c r="U14" s="6">
-        <v>999</v>
-      </c>
+      <c r="R14" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="S14" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="T14" s="6"/>
+      <c r="U14" s="6"/>
       <c r="V14" s="6"/>
       <c r="W14" s="6"/>
     </row>
     <row r="15" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E15" s="7">
         <v>60</v>
@@ -1388,55 +1419,52 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
+      <c r="H15" t="s">
+        <v>75</v>
+      </c>
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
-      <c r="L15" s="6">
-        <v>45</v>
-      </c>
-      <c r="M15" s="6">
-        <v>49</v>
-      </c>
-      <c r="N15" s="6">
+      <c r="L15" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O15" s="6">
+      <c r="M15" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N15" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O15" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P15" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q15" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P15" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q15" s="6">
-        <v>71</v>
-      </c>
-      <c r="R15" s="6">
-        <v>76</v>
-      </c>
-      <c r="S15" s="6">
-        <v>81</v>
-      </c>
-      <c r="T15" s="6">
-        <v>87</v>
-      </c>
-      <c r="U15" s="6">
-        <v>999</v>
-      </c>
+      <c r="R15" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="S15" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="T15" s="6"/>
+      <c r="U15" s="6"/>
       <c r="V15" s="6"/>
       <c r="W15" s="6"/>
     </row>
     <row r="16" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E16" s="7">
         <v>65</v>
@@ -1448,55 +1476,52 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
+      <c r="H16" t="s">
+        <v>75</v>
+      </c>
       <c r="J16" s="6"/>
       <c r="K16" s="6"/>
-      <c r="L16" s="6">
-        <v>45</v>
-      </c>
-      <c r="M16" s="6">
-        <v>49</v>
-      </c>
-      <c r="N16" s="6">
+      <c r="L16" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O16" s="6">
+      <c r="M16" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N16" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O16" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P16" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q16" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P16" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q16" s="6">
-        <v>71</v>
-      </c>
-      <c r="R16" s="6">
-        <v>76</v>
-      </c>
-      <c r="S16" s="6">
-        <v>81</v>
-      </c>
-      <c r="T16" s="6">
-        <v>87</v>
-      </c>
-      <c r="U16" s="6">
-        <v>999</v>
-      </c>
+      <c r="R16" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="S16" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="T16" s="6"/>
+      <c r="U16" s="6"/>
       <c r="V16" s="6"/>
       <c r="W16" s="6"/>
     </row>
     <row r="17" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E17" s="7">
         <v>70</v>
@@ -1508,55 +1533,52 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
+      <c r="H17" t="s">
+        <v>75</v>
+      </c>
       <c r="J17" s="6"/>
       <c r="K17" s="6"/>
-      <c r="L17" s="6">
-        <v>45</v>
-      </c>
-      <c r="M17" s="6">
-        <v>49</v>
-      </c>
-      <c r="N17" s="6">
+      <c r="L17" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O17" s="6">
+      <c r="M17" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N17" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O17" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P17" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q17" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P17" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q17" s="6">
-        <v>71</v>
-      </c>
-      <c r="R17" s="6">
-        <v>76</v>
-      </c>
-      <c r="S17" s="6">
-        <v>81</v>
-      </c>
-      <c r="T17" s="6">
-        <v>87</v>
-      </c>
-      <c r="U17" s="6">
-        <v>999</v>
-      </c>
+      <c r="R17" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="S17" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="T17" s="6"/>
+      <c r="U17" s="6"/>
       <c r="V17" s="6"/>
       <c r="W17" s="6"/>
     </row>
     <row r="18" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E18" s="7">
         <v>75</v>
@@ -1568,55 +1590,52 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
+      <c r="H18" t="s">
+        <v>75</v>
+      </c>
       <c r="J18" s="6"/>
       <c r="K18" s="6"/>
-      <c r="L18" s="6">
-        <v>45</v>
-      </c>
-      <c r="M18" s="6">
-        <v>49</v>
-      </c>
-      <c r="N18" s="6">
+      <c r="L18" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O18" s="6">
+      <c r="M18" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N18" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O18" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P18" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q18" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P18" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q18" s="6">
-        <v>71</v>
-      </c>
-      <c r="R18" s="6">
-        <v>76</v>
-      </c>
-      <c r="S18" s="6">
-        <v>81</v>
-      </c>
-      <c r="T18" s="6">
-        <v>87</v>
-      </c>
-      <c r="U18" s="6">
-        <v>999</v>
-      </c>
+      <c r="R18" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="S18" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="T18" s="6"/>
+      <c r="U18" s="6"/>
       <c r="V18" s="6"/>
       <c r="W18" s="6"/>
     </row>
     <row r="19" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E19" s="7">
         <v>80</v>
@@ -1628,55 +1647,52 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
+      <c r="H19" t="s">
+        <v>75</v>
+      </c>
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
-      <c r="L19" s="6">
-        <v>45</v>
-      </c>
-      <c r="M19" s="6">
-        <v>49</v>
-      </c>
-      <c r="N19" s="6">
+      <c r="L19" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O19" s="6">
+      <c r="M19" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N19" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O19" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P19" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q19" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P19" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q19" s="6">
-        <v>71</v>
-      </c>
-      <c r="R19" s="6">
-        <v>76</v>
-      </c>
-      <c r="S19" s="6">
-        <v>81</v>
-      </c>
-      <c r="T19" s="6">
-        <v>87</v>
-      </c>
-      <c r="U19" s="6">
-        <v>999</v>
-      </c>
+      <c r="R19" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="S19" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="T19" s="6"/>
+      <c r="U19" s="6"/>
       <c r="V19" s="6"/>
       <c r="W19" s="6"/>
     </row>
     <row r="20" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E20" s="10">
         <v>85</v>
@@ -1688,40 +1704,37 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H20" s="11"/>
-      <c r="I20" s="8"/>
+      <c r="H20" t="s">
+        <v>75</v>
+      </c>
       <c r="J20" s="12"/>
       <c r="K20" s="12"/>
-      <c r="L20" s="12">
-        <v>45</v>
-      </c>
-      <c r="M20" s="12">
-        <v>49</v>
-      </c>
-      <c r="N20" s="12">
+      <c r="L20" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O20" s="12">
+      <c r="M20" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N20" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O20" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P20" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q20" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P20" s="12">
-        <v>64</v>
-      </c>
-      <c r="Q20" s="12">
-        <v>71</v>
-      </c>
-      <c r="R20" s="12">
-        <v>76</v>
-      </c>
-      <c r="S20" s="12">
-        <v>81</v>
-      </c>
-      <c r="T20" s="12">
-        <v>87</v>
-      </c>
-      <c r="U20" s="12">
-        <v>999</v>
-      </c>
+      <c r="R20" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="S20" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="T20" s="12"/>
+      <c r="U20" s="12"/>
       <c r="V20" s="12"/>
       <c r="W20" s="12"/>
       <c r="X20" s="13"/>
@@ -1732,16 +1745,16 @@
     </row>
     <row r="21" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="D21" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E21" s="7">
         <v>13</v>
@@ -1753,55 +1766,52 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
+      <c r="H21" t="s">
+        <v>75</v>
+      </c>
       <c r="J21" s="6"/>
-      <c r="K21" s="6">
-        <v>40</v>
-      </c>
-      <c r="L21" s="6">
-        <v>45</v>
-      </c>
-      <c r="M21" s="6">
-        <v>49</v>
-      </c>
-      <c r="N21" s="6">
+      <c r="K21" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="L21" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O21" s="6">
+      <c r="M21" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N21" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O21" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P21" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q21" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P21" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q21" s="6">
-        <v>71</v>
-      </c>
-      <c r="R21" s="6">
-        <v>76</v>
-      </c>
-      <c r="S21" s="6">
-        <v>81</v>
-      </c>
-      <c r="T21" s="6">
-        <v>999</v>
-      </c>
+      <c r="R21" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="S21" s="6"/>
+      <c r="T21" s="6"/>
       <c r="U21" s="6"/>
       <c r="V21" s="6"/>
       <c r="W21" s="6"/>
     </row>
     <row r="22" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E22" s="7">
         <v>15</v>
@@ -1813,55 +1823,52 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
+      <c r="H22" t="s">
+        <v>75</v>
+      </c>
       <c r="J22" s="6"/>
       <c r="K22" s="6"/>
-      <c r="L22" s="6">
-        <v>45</v>
-      </c>
-      <c r="M22" s="6">
-        <v>49</v>
-      </c>
-      <c r="N22" s="6">
+      <c r="L22" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O22" s="6">
+      <c r="M22" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N22" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O22" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P22" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q22" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P22" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q22" s="6">
-        <v>71</v>
-      </c>
-      <c r="R22" s="6">
-        <v>76</v>
-      </c>
-      <c r="S22" s="6">
-        <v>81</v>
-      </c>
-      <c r="T22" s="6">
-        <v>87</v>
-      </c>
-      <c r="U22" s="6">
-        <v>999</v>
-      </c>
+      <c r="R22" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="S22" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="T22" s="6"/>
+      <c r="U22" s="6"/>
       <c r="V22" s="6"/>
       <c r="W22" s="6"/>
     </row>
     <row r="23" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E23" s="7">
         <v>15</v>
@@ -1873,55 +1880,52 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
+      <c r="H23" t="s">
+        <v>75</v>
+      </c>
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
-      <c r="L23" s="6">
-        <v>45</v>
-      </c>
-      <c r="M23" s="6">
-        <v>49</v>
-      </c>
-      <c r="N23" s="6">
+      <c r="L23" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O23" s="6">
+      <c r="M23" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N23" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O23" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P23" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q23" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P23" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q23" s="6">
-        <v>71</v>
-      </c>
-      <c r="R23" s="6">
-        <v>76</v>
-      </c>
-      <c r="S23" s="6">
-        <v>81</v>
-      </c>
-      <c r="T23" s="6">
-        <v>87</v>
-      </c>
-      <c r="U23" s="6">
-        <v>999</v>
-      </c>
+      <c r="R23" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="S23" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="T23" s="6"/>
+      <c r="U23" s="6"/>
       <c r="V23" s="6"/>
       <c r="W23" s="6"/>
     </row>
     <row r="24" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E24" s="7">
         <v>0</v>
@@ -1933,59 +1937,56 @@
         <f>TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
-      <c r="J24" s="6">
-        <v>35</v>
-      </c>
-      <c r="K24" s="6">
-        <v>40</v>
-      </c>
-      <c r="L24" s="6">
-        <v>45</v>
-      </c>
-      <c r="M24" s="6">
-        <v>49</v>
-      </c>
-      <c r="N24" s="6">
+      <c r="H24" t="s">
+        <v>75</v>
+      </c>
+      <c r="J24" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="L24" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O24" s="6">
+      <c r="M24" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N24" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O24" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="P24" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q24" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P24" s="6">
-        <v>64</v>
-      </c>
-      <c r="Q24" s="6">
-        <v>71</v>
-      </c>
-      <c r="R24" s="6">
-        <v>76</v>
-      </c>
-      <c r="S24" s="6">
-        <v>81</v>
-      </c>
-      <c r="T24" s="6">
-        <v>87</v>
-      </c>
-      <c r="U24" s="6">
-        <v>999</v>
-      </c>
+      <c r="R24" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="S24" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="T24" s="6"/>
+      <c r="U24" s="6"/>
       <c r="V24" s="6"/>
       <c r="W24" s="6"/>
     </row>
     <row r="25" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E25" s="7">
         <v>0</v>
@@ -1996,13 +1997,10 @@
       <c r="G25" s="8" t="b">
         <v>0</v>
       </c>
-      <c r="H25" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="I25" s="8"/>
-      <c r="J25" s="6" t="s">
-        <v>53</v>
-      </c>
+      <c r="H25" t="s">
+        <v>76</v>
+      </c>
+      <c r="J25" s="6"/>
       <c r="K25" s="6"/>
       <c r="L25" s="6"/>
       <c r="M25" s="6"/>
@@ -2015,62 +2013,73 @@
       <c r="T25" s="6"/>
       <c r="U25" s="6"/>
       <c r="V25" s="6"/>
-      <c r="W25" s="6"/>
     </row>
     <row r="26" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E26" s="7">
         <v>0</v>
       </c>
       <c r="F26" s="7">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G26" s="8" t="b">
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H26" s="8"/>
-      <c r="I26" s="8"/>
-      <c r="J26" s="6">
-        <v>999</v>
-      </c>
-      <c r="K26" s="6"/>
-      <c r="L26" s="6"/>
-      <c r="M26" s="6"/>
-      <c r="N26" s="6"/>
-      <c r="O26" s="6"/>
-      <c r="P26" s="6"/>
+      <c r="H26" t="s">
+        <v>75</v>
+      </c>
+      <c r="J26" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="L26" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="M26" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N26" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O26" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P26" s="6" t="s">
+        <v>51</v>
+      </c>
       <c r="Q26" s="6"/>
       <c r="R26" s="6"/>
       <c r="S26" s="6"/>
       <c r="T26" s="6"/>
       <c r="U26" s="6"/>
       <c r="V26" s="6"/>
-      <c r="W26" s="6"/>
     </row>
     <row r="27" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E27" s="7">
         <v>11</v>
@@ -2082,53 +2091,51 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H27" s="8"/>
-      <c r="I27" s="8"/>
-      <c r="J27" s="6">
-        <v>35</v>
-      </c>
-      <c r="K27" s="6">
-        <v>40</v>
-      </c>
-      <c r="L27" s="6">
-        <v>45</v>
-      </c>
-      <c r="M27" s="6">
-        <v>49</v>
-      </c>
-      <c r="N27" s="6">
+      <c r="H27" t="s">
+        <v>75</v>
+      </c>
+      <c r="J27" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="K27" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O27" s="6">
-        <v>61</v>
-      </c>
-      <c r="P27" s="6">
+      <c r="L27" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="M27" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N27" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O27" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P27" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q27" s="6">
-        <v>73</v>
-      </c>
-      <c r="R27" s="6">
-        <v>999</v>
-      </c>
+      <c r="Q27" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="R27" s="6"/>
       <c r="S27" s="6"/>
       <c r="T27" s="6"/>
       <c r="U27" s="6"/>
       <c r="V27" s="6"/>
-      <c r="W27" s="6"/>
     </row>
     <row r="28" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E28" s="7">
         <v>14</v>
@@ -2140,54 +2147,50 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H28" s="8"/>
-      <c r="I28" s="8"/>
+      <c r="H28" t="s">
+        <v>75</v>
+      </c>
       <c r="J28" s="6"/>
-      <c r="K28" s="6">
-        <v>40</v>
-      </c>
-      <c r="L28" s="6">
-        <v>45</v>
-      </c>
-      <c r="M28" s="6">
-        <v>49</v>
-      </c>
-      <c r="N28" s="6">
-        <v>55</v>
-      </c>
-      <c r="O28" s="6">
-        <v>61</v>
-      </c>
-      <c r="P28" s="6">
+      <c r="K28" s="6"/>
+      <c r="L28" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="M28" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N28" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O28" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P28" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q28" s="6">
-        <v>73</v>
+      <c r="Q28" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R28" s="6">
-        <v>81</v>
-      </c>
-      <c r="S28" s="6">
-        <v>89</v>
-      </c>
-      <c r="T28" s="6">
-        <v>999</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="S28" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U28" s="6"/>
       <c r="V28" s="6"/>
-      <c r="W28" s="6"/>
     </row>
     <row r="29" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E29" s="7">
         <v>16</v>
@@ -2199,54 +2202,50 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H29" s="8"/>
-      <c r="I29" s="8"/>
+      <c r="H29" t="s">
+        <v>75</v>
+      </c>
       <c r="J29" s="6"/>
       <c r="K29" s="6"/>
-      <c r="L29" s="6">
-        <v>45</v>
-      </c>
-      <c r="M29" s="6">
-        <v>49</v>
-      </c>
-      <c r="N29" s="6">
-        <v>55</v>
-      </c>
-      <c r="O29" s="6">
-        <v>61</v>
-      </c>
-      <c r="P29" s="6">
+      <c r="L29" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="M29" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N29" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O29" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P29" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q29" s="6">
-        <v>73</v>
+      <c r="Q29" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R29" s="6">
-        <v>81</v>
-      </c>
-      <c r="S29" s="6">
-        <v>89</v>
-      </c>
-      <c r="T29" s="6">
-        <v>96</v>
-      </c>
-      <c r="U29" s="6">
-        <v>999</v>
-      </c>
-      <c r="W29" s="6"/>
+        <v>94</v>
+      </c>
+      <c r="S29" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="T29" s="6"/>
+      <c r="V29" s="6"/>
     </row>
     <row r="30" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E30" s="7">
         <v>18</v>
@@ -2258,115 +2257,107 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H30" s="8"/>
-      <c r="I30" s="8"/>
+      <c r="H30" t="s">
+        <v>75</v>
+      </c>
       <c r="J30" s="6"/>
       <c r="K30" s="6"/>
       <c r="L30" s="6"/>
-      <c r="M30" s="6"/>
-      <c r="N30" s="6">
-        <v>55</v>
-      </c>
-      <c r="O30" s="6">
-        <v>61</v>
-      </c>
-      <c r="P30" s="6">
+      <c r="M30" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N30" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O30" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P30" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q30" s="6">
-        <v>73</v>
+      <c r="Q30" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R30" s="6">
-        <v>81</v>
-      </c>
-      <c r="S30" s="6">
-        <v>89</v>
-      </c>
-      <c r="T30" s="6">
-        <v>96</v>
-      </c>
-      <c r="U30" s="6">
-        <v>102</v>
-      </c>
-      <c r="V30" s="6">
-        <v>109</v>
-      </c>
-      <c r="W30" s="6">
-        <v>999</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="S30" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="T30" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U30" s="6"/>
+      <c r="V30" s="6"/>
     </row>
     <row r="31" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E31" s="7">
         <v>21</v>
       </c>
       <c r="F31" s="7">
-        <v>99</v>
+        <v>23</v>
       </c>
       <c r="G31" s="8" t="b">
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H31" s="8"/>
-      <c r="I31" s="8"/>
+      <c r="H31" t="s">
+        <v>75</v>
+      </c>
       <c r="J31" s="6"/>
       <c r="K31" s="6"/>
       <c r="L31" s="6"/>
-      <c r="M31" s="6"/>
-      <c r="N31" s="6">
-        <v>55</v>
-      </c>
-      <c r="O31" s="6">
-        <v>61</v>
-      </c>
-      <c r="P31" s="6">
+      <c r="M31" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N31" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O31" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P31" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q31" s="6">
-        <v>73</v>
+      <c r="Q31" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R31" s="6">
-        <v>81</v>
-      </c>
-      <c r="S31" s="6">
-        <v>89</v>
-      </c>
-      <c r="T31" s="6">
-        <v>96</v>
-      </c>
-      <c r="U31" s="6">
-        <v>102</v>
-      </c>
-      <c r="V31" s="6">
-        <v>109</v>
-      </c>
-      <c r="W31" s="6">
-        <v>999</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="S31" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="T31" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U31" s="6"/>
+      <c r="V31" s="6"/>
     </row>
     <row r="32" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E32" s="7">
         <v>30</v>
@@ -2378,55 +2369,51 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H32" s="8"/>
-      <c r="I32" s="8"/>
+      <c r="H32" t="s">
+        <v>75</v>
+      </c>
       <c r="J32" s="6"/>
       <c r="K32" s="6"/>
       <c r="L32" s="6"/>
-      <c r="M32" s="6"/>
-      <c r="N32" s="6">
-        <v>55</v>
-      </c>
-      <c r="O32" s="6">
-        <v>61</v>
-      </c>
-      <c r="P32" s="6">
+      <c r="M32" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N32" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O32" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P32" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q32" s="6">
-        <v>73</v>
+      <c r="Q32" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R32" s="6">
-        <v>81</v>
-      </c>
-      <c r="S32" s="6">
-        <v>89</v>
-      </c>
-      <c r="T32" s="6">
-        <v>96</v>
-      </c>
-      <c r="U32" s="6">
-        <v>102</v>
-      </c>
-      <c r="V32" s="6">
-        <v>109</v>
-      </c>
-      <c r="W32" s="6">
-        <v>999</v>
-      </c>
-    </row>
-    <row r="33" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+      <c r="S32" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="T32" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U32" s="6"/>
+      <c r="V32" s="6"/>
+    </row>
+    <row r="33" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E33" s="7">
         <v>35</v>
@@ -2438,55 +2425,51 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H33" s="8"/>
-      <c r="I33" s="8"/>
+      <c r="H33" t="s">
+        <v>75</v>
+      </c>
       <c r="J33" s="6"/>
       <c r="K33" s="6"/>
       <c r="L33" s="6"/>
-      <c r="M33" s="6"/>
-      <c r="N33" s="6">
-        <v>55</v>
-      </c>
-      <c r="O33" s="6">
-        <v>61</v>
-      </c>
-      <c r="P33" s="6">
+      <c r="M33" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N33" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O33" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P33" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q33" s="6">
-        <v>73</v>
+      <c r="Q33" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R33" s="6">
-        <v>81</v>
-      </c>
-      <c r="S33" s="6">
-        <v>89</v>
-      </c>
-      <c r="T33" s="6">
-        <v>96</v>
-      </c>
-      <c r="U33" s="6">
-        <v>102</v>
-      </c>
-      <c r="V33" s="6">
-        <v>109</v>
-      </c>
-      <c r="W33" s="6">
-        <v>999</v>
-      </c>
-    </row>
-    <row r="34" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+      <c r="S33" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="T33" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U33" s="6"/>
+      <c r="V33" s="6"/>
+    </row>
+    <row r="34" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E34" s="7">
         <v>40</v>
@@ -2498,55 +2481,51 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H34" s="8"/>
-      <c r="I34" s="8"/>
+      <c r="H34" t="s">
+        <v>75</v>
+      </c>
       <c r="J34" s="6"/>
       <c r="K34" s="6"/>
       <c r="L34" s="6"/>
-      <c r="M34" s="6"/>
-      <c r="N34" s="6">
-        <v>55</v>
-      </c>
-      <c r="O34" s="6">
-        <v>61</v>
-      </c>
-      <c r="P34" s="6">
+      <c r="M34" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N34" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O34" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P34" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q34" s="6">
-        <v>73</v>
+      <c r="Q34" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R34" s="6">
-        <v>81</v>
-      </c>
-      <c r="S34" s="6">
-        <v>89</v>
-      </c>
-      <c r="T34" s="6">
-        <v>96</v>
-      </c>
-      <c r="U34" s="6">
-        <v>102</v>
-      </c>
-      <c r="V34" s="6">
-        <v>109</v>
-      </c>
-      <c r="W34" s="6">
-        <v>999</v>
-      </c>
-    </row>
-    <row r="35" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+      <c r="S34" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="T34" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U34" s="6"/>
+      <c r="V34" s="6"/>
+    </row>
+    <row r="35" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E35" s="7">
         <v>45</v>
@@ -2558,55 +2537,51 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H35" s="8"/>
-      <c r="I35" s="8"/>
+      <c r="H35" t="s">
+        <v>75</v>
+      </c>
       <c r="J35" s="6"/>
       <c r="K35" s="6"/>
       <c r="L35" s="6"/>
-      <c r="M35" s="6"/>
-      <c r="N35" s="6">
-        <v>55</v>
-      </c>
-      <c r="O35" s="6">
-        <v>61</v>
-      </c>
-      <c r="P35" s="6">
+      <c r="M35" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N35" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O35" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P35" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q35" s="6">
-        <v>73</v>
+      <c r="Q35" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R35" s="6">
-        <v>81</v>
-      </c>
-      <c r="S35" s="6">
-        <v>89</v>
-      </c>
-      <c r="T35" s="6">
-        <v>96</v>
-      </c>
-      <c r="U35" s="6">
-        <v>102</v>
-      </c>
-      <c r="V35" s="6">
-        <v>109</v>
-      </c>
-      <c r="W35" s="6">
-        <v>999</v>
-      </c>
-    </row>
-    <row r="36" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+      <c r="S35" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="T35" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U35" s="6"/>
+      <c r="V35" s="6"/>
+    </row>
+    <row r="36" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E36" s="7">
         <v>50</v>
@@ -2618,55 +2593,51 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H36" s="8"/>
-      <c r="I36" s="8"/>
+      <c r="H36" t="s">
+        <v>75</v>
+      </c>
       <c r="J36" s="6"/>
       <c r="K36" s="6"/>
       <c r="L36" s="6"/>
-      <c r="M36" s="6"/>
-      <c r="N36" s="6">
-        <v>55</v>
-      </c>
-      <c r="O36" s="6">
-        <v>61</v>
-      </c>
-      <c r="P36" s="6">
+      <c r="M36" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N36" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O36" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P36" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q36" s="6">
-        <v>73</v>
+      <c r="Q36" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R36" s="6">
-        <v>81</v>
-      </c>
-      <c r="S36" s="6">
-        <v>89</v>
-      </c>
-      <c r="T36" s="6">
-        <v>96</v>
-      </c>
-      <c r="U36" s="6">
-        <v>102</v>
-      </c>
-      <c r="V36" s="6">
-        <v>109</v>
-      </c>
-      <c r="W36" s="6">
-        <v>999</v>
-      </c>
-    </row>
-    <row r="37" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+      <c r="S36" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="T36" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U36" s="6"/>
+      <c r="V36" s="6"/>
+    </row>
+    <row r="37" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E37" s="7">
         <v>55</v>
@@ -2678,55 +2649,51 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H37" s="8"/>
-      <c r="I37" s="8"/>
+      <c r="H37" t="s">
+        <v>75</v>
+      </c>
       <c r="J37" s="6"/>
       <c r="K37" s="6"/>
       <c r="L37" s="6"/>
-      <c r="M37" s="6"/>
-      <c r="N37" s="6">
-        <v>55</v>
-      </c>
-      <c r="O37" s="6">
-        <v>61</v>
-      </c>
-      <c r="P37" s="6">
+      <c r="M37" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N37" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O37" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P37" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q37" s="6">
-        <v>73</v>
+      <c r="Q37" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R37" s="6">
-        <v>81</v>
-      </c>
-      <c r="S37" s="6">
-        <v>89</v>
-      </c>
-      <c r="T37" s="6">
-        <v>96</v>
-      </c>
-      <c r="U37" s="6">
-        <v>102</v>
-      </c>
-      <c r="V37" s="6">
-        <v>109</v>
-      </c>
-      <c r="W37" s="6">
-        <v>999</v>
-      </c>
-    </row>
-    <row r="38" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+      <c r="S37" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="T37" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U37" s="6"/>
+      <c r="V37" s="6"/>
+    </row>
+    <row r="38" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E38" s="7">
         <v>60</v>
@@ -2738,55 +2705,51 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H38" s="8"/>
-      <c r="I38" s="8"/>
+      <c r="H38" t="s">
+        <v>75</v>
+      </c>
       <c r="J38" s="6"/>
       <c r="K38" s="6"/>
       <c r="L38" s="6"/>
-      <c r="M38" s="6"/>
-      <c r="N38" s="6">
-        <v>55</v>
-      </c>
-      <c r="O38" s="6">
-        <v>61</v>
-      </c>
-      <c r="P38" s="6">
+      <c r="M38" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N38" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O38" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P38" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q38" s="6">
-        <v>73</v>
+      <c r="Q38" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R38" s="6">
-        <v>81</v>
-      </c>
-      <c r="S38" s="6">
-        <v>89</v>
-      </c>
-      <c r="T38" s="6">
-        <v>96</v>
-      </c>
-      <c r="U38" s="6">
-        <v>102</v>
-      </c>
-      <c r="V38" s="6">
-        <v>109</v>
-      </c>
-      <c r="W38" s="6">
-        <v>999</v>
-      </c>
-    </row>
-    <row r="39" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+      <c r="S38" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="T38" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U38" s="6"/>
+      <c r="V38" s="6"/>
+    </row>
+    <row r="39" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E39" s="7">
         <v>65</v>
@@ -2798,55 +2761,51 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H39" s="8"/>
-      <c r="I39" s="8"/>
+      <c r="H39" t="s">
+        <v>75</v>
+      </c>
       <c r="J39" s="6"/>
       <c r="K39" s="6"/>
       <c r="L39" s="6"/>
-      <c r="M39" s="6"/>
-      <c r="N39" s="6">
-        <v>55</v>
-      </c>
-      <c r="O39" s="6">
-        <v>61</v>
-      </c>
-      <c r="P39" s="6">
+      <c r="M39" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N39" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O39" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P39" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q39" s="6">
-        <v>73</v>
+      <c r="Q39" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R39" s="6">
-        <v>81</v>
-      </c>
-      <c r="S39" s="6">
-        <v>89</v>
-      </c>
-      <c r="T39" s="6">
-        <v>96</v>
-      </c>
-      <c r="U39" s="6">
-        <v>102</v>
-      </c>
-      <c r="V39" s="6">
-        <v>109</v>
-      </c>
-      <c r="W39" s="6">
-        <v>999</v>
-      </c>
-    </row>
-    <row r="40" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+      <c r="S39" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="T39" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U39" s="6"/>
+      <c r="V39" s="6"/>
+    </row>
+    <row r="40" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E40" s="7">
         <v>70</v>
@@ -2858,55 +2817,51 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H40" s="8"/>
-      <c r="I40" s="8"/>
+      <c r="H40" t="s">
+        <v>75</v>
+      </c>
       <c r="J40" s="6"/>
       <c r="K40" s="6"/>
       <c r="L40" s="6"/>
-      <c r="M40" s="6"/>
-      <c r="N40" s="6">
-        <v>55</v>
-      </c>
-      <c r="O40" s="6">
-        <v>61</v>
-      </c>
-      <c r="P40" s="6">
+      <c r="M40" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N40" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O40" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P40" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q40" s="6">
-        <v>73</v>
+      <c r="Q40" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R40" s="6">
-        <v>81</v>
-      </c>
-      <c r="S40" s="6">
-        <v>89</v>
-      </c>
-      <c r="T40" s="6">
-        <v>96</v>
-      </c>
-      <c r="U40" s="6">
-        <v>102</v>
-      </c>
-      <c r="V40" s="6">
-        <v>109</v>
-      </c>
-      <c r="W40" s="6">
-        <v>999</v>
-      </c>
-    </row>
-    <row r="41" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+      <c r="S40" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="T40" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U40" s="6"/>
+      <c r="V40" s="6"/>
+    </row>
+    <row r="41" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E41" s="7">
         <v>75</v>
@@ -2918,55 +2873,51 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H41" s="8"/>
-      <c r="I41" s="8"/>
+      <c r="H41" t="s">
+        <v>75</v>
+      </c>
       <c r="J41" s="6"/>
       <c r="K41" s="6"/>
       <c r="L41" s="6"/>
-      <c r="M41" s="6"/>
-      <c r="N41" s="6">
-        <v>55</v>
-      </c>
-      <c r="O41" s="6">
-        <v>61</v>
-      </c>
-      <c r="P41" s="6">
+      <c r="M41" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N41" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O41" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P41" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q41" s="6">
-        <v>73</v>
+      <c r="Q41" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R41" s="6">
-        <v>81</v>
-      </c>
-      <c r="S41" s="6">
-        <v>89</v>
-      </c>
-      <c r="T41" s="6">
-        <v>96</v>
-      </c>
-      <c r="U41" s="6">
-        <v>102</v>
-      </c>
-      <c r="V41" s="6">
-        <v>109</v>
-      </c>
-      <c r="W41" s="6">
-        <v>999</v>
-      </c>
-    </row>
-    <row r="42" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+      <c r="S41" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="T41" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U41" s="6"/>
+      <c r="V41" s="6"/>
+    </row>
+    <row r="42" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E42" s="7">
         <v>80</v>
@@ -2978,55 +2929,51 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H42" s="8"/>
-      <c r="I42" s="8"/>
+      <c r="H42" t="s">
+        <v>75</v>
+      </c>
       <c r="J42" s="6"/>
       <c r="K42" s="6"/>
       <c r="L42" s="6"/>
-      <c r="M42" s="6"/>
-      <c r="N42" s="6">
-        <v>55</v>
-      </c>
-      <c r="O42" s="6">
-        <v>61</v>
-      </c>
-      <c r="P42" s="6">
+      <c r="M42" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N42" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O42" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P42" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q42" s="6">
-        <v>73</v>
+      <c r="Q42" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R42" s="6">
-        <v>81</v>
-      </c>
-      <c r="S42" s="6">
-        <v>89</v>
-      </c>
-      <c r="T42" s="6">
-        <v>96</v>
-      </c>
-      <c r="U42" s="6">
-        <v>102</v>
-      </c>
-      <c r="V42" s="6">
-        <v>109</v>
-      </c>
-      <c r="W42" s="6">
-        <v>999</v>
-      </c>
-    </row>
-    <row r="43" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+      <c r="S42" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="T42" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U42" s="6"/>
+      <c r="V42" s="6"/>
+    </row>
+    <row r="43" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E43" s="7">
         <v>85</v>
@@ -3038,55 +2985,51 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H43" s="8"/>
-      <c r="I43" s="8"/>
+      <c r="H43" t="s">
+        <v>75</v>
+      </c>
       <c r="J43" s="6"/>
       <c r="K43" s="6"/>
       <c r="L43" s="6"/>
-      <c r="M43" s="6"/>
-      <c r="N43" s="6">
-        <v>55</v>
-      </c>
-      <c r="O43" s="6">
-        <v>61</v>
-      </c>
-      <c r="P43" s="6">
+      <c r="M43" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N43" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O43" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P43" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q43" s="6">
-        <v>73</v>
+      <c r="Q43" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R43" s="6">
-        <v>81</v>
-      </c>
-      <c r="S43" s="6">
-        <v>89</v>
-      </c>
-      <c r="T43" s="6">
-        <v>96</v>
-      </c>
-      <c r="U43" s="6">
-        <v>102</v>
-      </c>
-      <c r="V43" s="6">
-        <v>109</v>
-      </c>
-      <c r="W43" s="6">
-        <v>999</v>
-      </c>
-    </row>
-    <row r="44" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+      <c r="S43" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="T43" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U43" s="6"/>
+      <c r="V43" s="6"/>
+    </row>
+    <row r="44" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B44" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="D44" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E44" s="7">
         <v>13</v>
@@ -3098,55 +3041,51 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H44" s="8"/>
-      <c r="I44" s="8"/>
+      <c r="H44" t="s">
+        <v>75</v>
+      </c>
       <c r="J44" s="6"/>
       <c r="K44" s="6"/>
-      <c r="L44" s="6"/>
-      <c r="M44" s="6">
-        <v>49</v>
-      </c>
-      <c r="N44" s="6">
-        <v>55</v>
-      </c>
-      <c r="O44" s="6">
-        <v>61</v>
-      </c>
-      <c r="P44" s="6">
+      <c r="L44" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="M44" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N44" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O44" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P44" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q44" s="6">
-        <v>73</v>
+      <c r="Q44" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R44" s="6">
-        <v>81</v>
-      </c>
-      <c r="S44" s="6">
-        <v>89</v>
-      </c>
-      <c r="T44" s="6">
-        <v>96</v>
-      </c>
-      <c r="U44" s="6">
-        <v>102</v>
-      </c>
-      <c r="V44" s="6">
-        <v>999</v>
-      </c>
-      <c r="W44" s="6"/>
-    </row>
-    <row r="45" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+      <c r="S44" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="T44" s="6"/>
+      <c r="U44" s="6"/>
+      <c r="V44" s="6"/>
+    </row>
+    <row r="45" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E45" s="7">
         <v>15</v>
@@ -3158,55 +3097,51 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H45" s="8"/>
-      <c r="I45" s="8"/>
+      <c r="H45" t="s">
+        <v>75</v>
+      </c>
       <c r="J45" s="6"/>
       <c r="K45" s="6"/>
       <c r="L45" s="6"/>
-      <c r="M45" s="6"/>
-      <c r="N45" s="6">
-        <v>55</v>
-      </c>
-      <c r="O45" s="6">
-        <v>61</v>
-      </c>
-      <c r="P45" s="6">
+      <c r="M45" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N45" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O45" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P45" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q45" s="6">
-        <v>73</v>
+      <c r="Q45" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R45" s="6">
-        <v>81</v>
-      </c>
-      <c r="S45" s="6">
-        <v>89</v>
-      </c>
-      <c r="T45" s="6">
-        <v>96</v>
-      </c>
-      <c r="U45" s="6">
-        <v>102</v>
-      </c>
-      <c r="V45" s="6">
-        <v>109</v>
-      </c>
-      <c r="W45" s="6">
-        <v>999</v>
-      </c>
-    </row>
-    <row r="46" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+      <c r="S45" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="T45" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U45" s="6"/>
+      <c r="V45" s="6"/>
+    </row>
+    <row r="46" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E46" s="7">
         <v>15</v>
@@ -3218,55 +3153,51 @@
         <f>FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H46" s="8"/>
-      <c r="I46" s="8"/>
+      <c r="H46" t="s">
+        <v>75</v>
+      </c>
       <c r="J46" s="6"/>
       <c r="K46" s="6"/>
       <c r="L46" s="6"/>
-      <c r="M46" s="6"/>
-      <c r="N46" s="6">
-        <v>55</v>
-      </c>
-      <c r="O46" s="6">
-        <v>61</v>
-      </c>
-      <c r="P46" s="6">
+      <c r="M46" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N46" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O46" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P46" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q46" s="6">
-        <v>73</v>
+      <c r="Q46" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R46" s="6">
-        <v>81</v>
-      </c>
-      <c r="S46" s="6">
-        <v>89</v>
-      </c>
-      <c r="T46" s="6">
-        <v>96</v>
-      </c>
-      <c r="U46" s="6">
-        <v>102</v>
-      </c>
-      <c r="V46" s="6">
-        <v>109</v>
-      </c>
-      <c r="W46" s="6">
-        <v>999</v>
-      </c>
-    </row>
-    <row r="47" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+      <c r="S46" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="T46" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U46" s="6"/>
+      <c r="V46" s="6"/>
+    </row>
+    <row r="47" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D47" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="E47" s="7">
         <v>0</v>
@@ -3278,52 +3209,46 @@
         <f>TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H47" s="8"/>
-      <c r="I47" s="8"/>
-      <c r="J47" s="6">
-        <v>35</v>
-      </c>
-      <c r="K47" s="6">
-        <v>40</v>
-      </c>
-      <c r="L47" s="6">
-        <v>45</v>
-      </c>
-      <c r="M47" s="6">
-        <v>49</v>
-      </c>
-      <c r="N47" s="6">
+      <c r="H47" t="s">
+        <v>75</v>
+      </c>
+      <c r="J47" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="K47" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="O47" s="6">
-        <v>61</v>
-      </c>
-      <c r="P47" s="6">
+      <c r="L47" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="M47" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N47" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O47" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="P47" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="Q47" s="6">
-        <v>73</v>
+      <c r="Q47" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="R47" s="6">
-        <v>81</v>
-      </c>
-      <c r="S47" s="6">
-        <v>89</v>
-      </c>
-      <c r="T47" s="6">
-        <v>96</v>
-      </c>
-      <c r="U47" s="6">
-        <v>102</v>
-      </c>
-      <c r="V47" s="6">
-        <v>109</v>
-      </c>
-      <c r="W47" s="6">
-        <v>999</v>
-      </c>
-    </row>
-    <row r="48" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+        <v>94</v>
+      </c>
+      <c r="S47" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="T47" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U47" s="6"/>
+      <c r="V47" s="6"/>
+    </row>
+    <row r="48" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="49" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="50" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="51" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>